<commit_message>
fix: update status of は vs が to READY in Excel sheet
</commit_message>
<xml_diff>
--- a/投稿アイデア管理シート.xlsx
+++ b/投稿アイデア管理シート.xlsx
@@ -566,7 +566,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -649,9 +649,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>PUBLISHED</t>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>READY</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -794,7 +794,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -1022,7 +1022,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
chore: mark は vs が as PUBLISHED
</commit_message>
<xml_diff>
--- a/投稿アイデア管理シート.xlsx
+++ b/投稿アイデア管理シート.xlsx
@@ -649,9 +649,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>READY</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">

</xml_diff>